<commit_message>
chore(data-release): publish site data 2026-10-31 05:06:11 UTC
</commit_message>
<xml_diff>
--- a/diseases/d001/1995-1999.xlsx
+++ b/diseases/d001/1995-1999.xlsx
@@ -1938,6 +1938,11 @@
       <c r="Q8" t="n">
         <v>0</v>
       </c>
+      <c r="S8" t="inlineStr">
+        <is>
+          <t>missing_population</t>
+        </is>
+      </c>
       <c r="AA8" t="inlineStr">
         <is>
           <t>monthly</t>
@@ -1950,12 +1955,22 @@
       </c>
       <c r="AP8" t="inlineStr">
         <is>
-          <t>published_series</t>
+          <t>legacy_fallback</t>
+        </is>
+      </c>
+      <c r="AR8" t="inlineStr">
+        <is>
+          <t>legacy_identity_may_be_lossy</t>
         </is>
       </c>
       <c r="AS8" t="inlineStr"/>
       <c r="AT8" t="n">
         <v>0</v>
+      </c>
+      <c r="AU8" t="inlineStr">
+        <is>
+          <t>No eligible registered case-count series facts are available for this disease and country; the public curve uses the legacy flat table.</t>
+        </is>
       </c>
       <c r="AV8" t="inlineStr">
         <is>
@@ -2312,6 +2327,11 @@
       <c r="Q10" t="n">
         <v>0</v>
       </c>
+      <c r="S10" t="inlineStr">
+        <is>
+          <t>missing_population</t>
+        </is>
+      </c>
       <c r="AA10" t="inlineStr">
         <is>
           <t>monthly</t>
@@ -2324,12 +2344,22 @@
       </c>
       <c r="AP10" t="inlineStr">
         <is>
-          <t>published_series</t>
+          <t>legacy_fallback</t>
+        </is>
+      </c>
+      <c r="AR10" t="inlineStr">
+        <is>
+          <t>legacy_identity_may_be_lossy</t>
         </is>
       </c>
       <c r="AS10" t="inlineStr"/>
       <c r="AT10" t="n">
         <v>0</v>
+      </c>
+      <c r="AU10" t="inlineStr">
+        <is>
+          <t>No eligible registered case-count series facts are available for this disease and country; the public curve uses the legacy flat table.</t>
+        </is>
       </c>
       <c r="AV10" t="inlineStr">
         <is>
@@ -2447,6 +2477,11 @@
       <c r="Q11" t="n">
         <v>0</v>
       </c>
+      <c r="S11" t="inlineStr">
+        <is>
+          <t>missing_population</t>
+        </is>
+      </c>
       <c r="AA11" t="inlineStr">
         <is>
           <t>monthly</t>
@@ -2459,12 +2494,22 @@
       </c>
       <c r="AP11" t="inlineStr">
         <is>
-          <t>published_series</t>
+          <t>legacy_fallback</t>
+        </is>
+      </c>
+      <c r="AR11" t="inlineStr">
+        <is>
+          <t>legacy_identity_may_be_lossy</t>
         </is>
       </c>
       <c r="AS11" t="inlineStr"/>
       <c r="AT11" t="n">
         <v>0</v>
+      </c>
+      <c r="AU11" t="inlineStr">
+        <is>
+          <t>No eligible registered case-count series facts are available for this disease and country; the public curve uses the legacy flat table.</t>
+        </is>
       </c>
       <c r="AV11" t="inlineStr">
         <is>
@@ -2582,6 +2627,11 @@
       <c r="Q12" t="n">
         <v>0</v>
       </c>
+      <c r="S12" t="inlineStr">
+        <is>
+          <t>missing_population</t>
+        </is>
+      </c>
       <c r="AA12" t="inlineStr">
         <is>
           <t>monthly</t>
@@ -2594,12 +2644,22 @@
       </c>
       <c r="AP12" t="inlineStr">
         <is>
-          <t>published_series</t>
+          <t>legacy_fallback</t>
+        </is>
+      </c>
+      <c r="AR12" t="inlineStr">
+        <is>
+          <t>legacy_identity_may_be_lossy</t>
         </is>
       </c>
       <c r="AS12" t="inlineStr"/>
       <c r="AT12" t="n">
         <v>0</v>
+      </c>
+      <c r="AU12" t="inlineStr">
+        <is>
+          <t>No eligible registered case-count series facts are available for this disease and country; the public curve uses the legacy flat table.</t>
+        </is>
       </c>
       <c r="AV12" t="inlineStr">
         <is>
@@ -2717,6 +2777,11 @@
       <c r="Q13" t="n">
         <v>0</v>
       </c>
+      <c r="S13" t="inlineStr">
+        <is>
+          <t>missing_population</t>
+        </is>
+      </c>
       <c r="AA13" t="inlineStr">
         <is>
           <t>monthly</t>
@@ -2729,12 +2794,22 @@
       </c>
       <c r="AP13" t="inlineStr">
         <is>
-          <t>published_series</t>
+          <t>legacy_fallback</t>
+        </is>
+      </c>
+      <c r="AR13" t="inlineStr">
+        <is>
+          <t>legacy_identity_may_be_lossy</t>
         </is>
       </c>
       <c r="AS13" t="inlineStr"/>
       <c r="AT13" t="n">
         <v>0</v>
+      </c>
+      <c r="AU13" t="inlineStr">
+        <is>
+          <t>No eligible registered case-count series facts are available for this disease and country; the public curve uses the legacy flat table.</t>
+        </is>
       </c>
       <c r="AV13" t="inlineStr">
         <is>
@@ -2852,6 +2927,11 @@
       <c r="Q14" t="n">
         <v>0</v>
       </c>
+      <c r="S14" t="inlineStr">
+        <is>
+          <t>missing_population</t>
+        </is>
+      </c>
       <c r="AA14" t="inlineStr">
         <is>
           <t>monthly</t>
@@ -2864,12 +2944,22 @@
       </c>
       <c r="AP14" t="inlineStr">
         <is>
-          <t>published_series</t>
+          <t>legacy_fallback</t>
+        </is>
+      </c>
+      <c r="AR14" t="inlineStr">
+        <is>
+          <t>legacy_identity_may_be_lossy</t>
         </is>
       </c>
       <c r="AS14" t="inlineStr"/>
       <c r="AT14" t="n">
         <v>0</v>
+      </c>
+      <c r="AU14" t="inlineStr">
+        <is>
+          <t>No eligible registered case-count series facts are available for this disease and country; the public curve uses the legacy flat table.</t>
+        </is>
       </c>
       <c r="AV14" t="inlineStr">
         <is>
@@ -2987,6 +3077,11 @@
       <c r="Q15" t="n">
         <v>0</v>
       </c>
+      <c r="S15" t="inlineStr">
+        <is>
+          <t>missing_population</t>
+        </is>
+      </c>
       <c r="AA15" t="inlineStr">
         <is>
           <t>monthly</t>
@@ -2999,12 +3094,22 @@
       </c>
       <c r="AP15" t="inlineStr">
         <is>
-          <t>published_series</t>
+          <t>legacy_fallback</t>
+        </is>
+      </c>
+      <c r="AR15" t="inlineStr">
+        <is>
+          <t>legacy_identity_may_be_lossy</t>
         </is>
       </c>
       <c r="AS15" t="inlineStr"/>
       <c r="AT15" t="n">
         <v>0</v>
+      </c>
+      <c r="AU15" t="inlineStr">
+        <is>
+          <t>No eligible registered case-count series facts are available for this disease and country; the public curve uses the legacy flat table.</t>
+        </is>
       </c>
       <c r="AV15" t="inlineStr">
         <is>
@@ -3122,6 +3227,11 @@
       <c r="Q16" t="n">
         <v>0</v>
       </c>
+      <c r="S16" t="inlineStr">
+        <is>
+          <t>missing_population</t>
+        </is>
+      </c>
       <c r="AA16" t="inlineStr">
         <is>
           <t>monthly</t>
@@ -3134,12 +3244,22 @@
       </c>
       <c r="AP16" t="inlineStr">
         <is>
-          <t>published_series</t>
+          <t>legacy_fallback</t>
+        </is>
+      </c>
+      <c r="AR16" t="inlineStr">
+        <is>
+          <t>legacy_identity_may_be_lossy</t>
         </is>
       </c>
       <c r="AS16" t="inlineStr"/>
       <c r="AT16" t="n">
         <v>0</v>
+      </c>
+      <c r="AU16" t="inlineStr">
+        <is>
+          <t>No eligible registered case-count series facts are available for this disease and country; the public curve uses the legacy flat table.</t>
+        </is>
       </c>
       <c r="AV16" t="inlineStr">
         <is>
@@ -3257,6 +3377,11 @@
       <c r="Q17" t="n">
         <v>0</v>
       </c>
+      <c r="S17" t="inlineStr">
+        <is>
+          <t>missing_population</t>
+        </is>
+      </c>
       <c r="AA17" t="inlineStr">
         <is>
           <t>monthly</t>
@@ -3269,12 +3394,22 @@
       </c>
       <c r="AP17" t="inlineStr">
         <is>
-          <t>published_series</t>
+          <t>legacy_fallback</t>
+        </is>
+      </c>
+      <c r="AR17" t="inlineStr">
+        <is>
+          <t>legacy_identity_may_be_lossy</t>
         </is>
       </c>
       <c r="AS17" t="inlineStr"/>
       <c r="AT17" t="n">
         <v>0</v>
+      </c>
+      <c r="AU17" t="inlineStr">
+        <is>
+          <t>No eligible registered case-count series facts are available for this disease and country; the public curve uses the legacy flat table.</t>
+        </is>
       </c>
       <c r="AV17" t="inlineStr">
         <is>
@@ -3392,6 +3527,11 @@
       <c r="Q18" t="n">
         <v>0</v>
       </c>
+      <c r="S18" t="inlineStr">
+        <is>
+          <t>missing_population</t>
+        </is>
+      </c>
       <c r="AA18" t="inlineStr">
         <is>
           <t>monthly</t>
@@ -3404,12 +3544,22 @@
       </c>
       <c r="AP18" t="inlineStr">
         <is>
-          <t>published_series</t>
+          <t>legacy_fallback</t>
+        </is>
+      </c>
+      <c r="AR18" t="inlineStr">
+        <is>
+          <t>legacy_identity_may_be_lossy</t>
         </is>
       </c>
       <c r="AS18" t="inlineStr"/>
       <c r="AT18" t="n">
         <v>0</v>
+      </c>
+      <c r="AU18" t="inlineStr">
+        <is>
+          <t>No eligible registered case-count series facts are available for this disease and country; the public curve uses the legacy flat table.</t>
+        </is>
       </c>
       <c r="AV18" t="inlineStr">
         <is>
@@ -3527,6 +3677,11 @@
       <c r="Q19" t="n">
         <v>0</v>
       </c>
+      <c r="S19" t="inlineStr">
+        <is>
+          <t>missing_population</t>
+        </is>
+      </c>
       <c r="AA19" t="inlineStr">
         <is>
           <t>monthly</t>
@@ -3539,12 +3694,22 @@
       </c>
       <c r="AP19" t="inlineStr">
         <is>
-          <t>published_series</t>
+          <t>legacy_fallback</t>
+        </is>
+      </c>
+      <c r="AR19" t="inlineStr">
+        <is>
+          <t>legacy_identity_may_be_lossy</t>
         </is>
       </c>
       <c r="AS19" t="inlineStr"/>
       <c r="AT19" t="n">
         <v>0</v>
+      </c>
+      <c r="AU19" t="inlineStr">
+        <is>
+          <t>No eligible registered case-count series facts are available for this disease and country; the public curve uses the legacy flat table.</t>
+        </is>
       </c>
       <c r="AV19" t="inlineStr">
         <is>
@@ -3662,6 +3827,11 @@
       <c r="Q20" t="n">
         <v>0</v>
       </c>
+      <c r="S20" t="inlineStr">
+        <is>
+          <t>missing_population</t>
+        </is>
+      </c>
       <c r="AA20" t="inlineStr">
         <is>
           <t>monthly</t>
@@ -3674,12 +3844,22 @@
       </c>
       <c r="AP20" t="inlineStr">
         <is>
-          <t>published_series</t>
+          <t>legacy_fallback</t>
+        </is>
+      </c>
+      <c r="AR20" t="inlineStr">
+        <is>
+          <t>legacy_identity_may_be_lossy</t>
         </is>
       </c>
       <c r="AS20" t="inlineStr"/>
       <c r="AT20" t="n">
         <v>0</v>
+      </c>
+      <c r="AU20" t="inlineStr">
+        <is>
+          <t>No eligible registered case-count series facts are available for this disease and country; the public curve uses the legacy flat table.</t>
+        </is>
       </c>
       <c r="AV20" t="inlineStr">
         <is>
@@ -4187,6 +4367,11 @@
       <c r="Q23" t="n">
         <v>0</v>
       </c>
+      <c r="S23" t="inlineStr">
+        <is>
+          <t>missing_population</t>
+        </is>
+      </c>
       <c r="AA23" t="inlineStr">
         <is>
           <t>monthly</t>
@@ -4199,12 +4384,22 @@
       </c>
       <c r="AP23" t="inlineStr">
         <is>
-          <t>published_series</t>
+          <t>legacy_fallback</t>
+        </is>
+      </c>
+      <c r="AR23" t="inlineStr">
+        <is>
+          <t>legacy_identity_may_be_lossy</t>
         </is>
       </c>
       <c r="AS23" t="inlineStr"/>
       <c r="AT23" t="n">
         <v>0</v>
+      </c>
+      <c r="AU23" t="inlineStr">
+        <is>
+          <t>No eligible registered case-count series facts are available for this disease and country; the public curve uses the legacy flat table.</t>
+        </is>
       </c>
       <c r="AV23" t="inlineStr">
         <is>
@@ -4561,6 +4756,11 @@
       <c r="Q25" t="n">
         <v>0</v>
       </c>
+      <c r="S25" t="inlineStr">
+        <is>
+          <t>missing_population</t>
+        </is>
+      </c>
       <c r="AA25" t="inlineStr">
         <is>
           <t>monthly</t>
@@ -4573,12 +4773,22 @@
       </c>
       <c r="AP25" t="inlineStr">
         <is>
-          <t>published_series</t>
+          <t>legacy_fallback</t>
+        </is>
+      </c>
+      <c r="AR25" t="inlineStr">
+        <is>
+          <t>legacy_identity_may_be_lossy</t>
         </is>
       </c>
       <c r="AS25" t="inlineStr"/>
       <c r="AT25" t="n">
         <v>0</v>
+      </c>
+      <c r="AU25" t="inlineStr">
+        <is>
+          <t>No eligible registered case-count series facts are available for this disease and country; the public curve uses the legacy flat table.</t>
+        </is>
       </c>
       <c r="AV25" t="inlineStr">
         <is>
@@ -4696,6 +4906,11 @@
       <c r="Q26" t="n">
         <v>0</v>
       </c>
+      <c r="S26" t="inlineStr">
+        <is>
+          <t>missing_population</t>
+        </is>
+      </c>
       <c r="AA26" t="inlineStr">
         <is>
           <t>monthly</t>
@@ -4708,12 +4923,22 @@
       </c>
       <c r="AP26" t="inlineStr">
         <is>
-          <t>published_series</t>
+          <t>legacy_fallback</t>
+        </is>
+      </c>
+      <c r="AR26" t="inlineStr">
+        <is>
+          <t>legacy_identity_may_be_lossy</t>
         </is>
       </c>
       <c r="AS26" t="inlineStr"/>
       <c r="AT26" t="n">
         <v>0</v>
+      </c>
+      <c r="AU26" t="inlineStr">
+        <is>
+          <t>No eligible registered case-count series facts are available for this disease and country; the public curve uses the legacy flat table.</t>
+        </is>
       </c>
       <c r="AV26" t="inlineStr">
         <is>
@@ -4831,6 +5056,11 @@
       <c r="Q27" t="n">
         <v>0</v>
       </c>
+      <c r="S27" t="inlineStr">
+        <is>
+          <t>missing_population</t>
+        </is>
+      </c>
       <c r="AA27" t="inlineStr">
         <is>
           <t>monthly</t>
@@ -4843,12 +5073,22 @@
       </c>
       <c r="AP27" t="inlineStr">
         <is>
-          <t>published_series</t>
+          <t>legacy_fallback</t>
+        </is>
+      </c>
+      <c r="AR27" t="inlineStr">
+        <is>
+          <t>legacy_identity_may_be_lossy</t>
         </is>
       </c>
       <c r="AS27" t="inlineStr"/>
       <c r="AT27" t="n">
         <v>0</v>
+      </c>
+      <c r="AU27" t="inlineStr">
+        <is>
+          <t>No eligible registered case-count series facts are available for this disease and country; the public curve uses the legacy flat table.</t>
+        </is>
       </c>
       <c r="AV27" t="inlineStr">
         <is>
@@ -4966,6 +5206,11 @@
       <c r="Q28" t="n">
         <v>0</v>
       </c>
+      <c r="S28" t="inlineStr">
+        <is>
+          <t>missing_population</t>
+        </is>
+      </c>
       <c r="AA28" t="inlineStr">
         <is>
           <t>monthly</t>
@@ -4978,12 +5223,22 @@
       </c>
       <c r="AP28" t="inlineStr">
         <is>
-          <t>published_series</t>
+          <t>legacy_fallback</t>
+        </is>
+      </c>
+      <c r="AR28" t="inlineStr">
+        <is>
+          <t>legacy_identity_may_be_lossy</t>
         </is>
       </c>
       <c r="AS28" t="inlineStr"/>
       <c r="AT28" t="n">
         <v>0</v>
+      </c>
+      <c r="AU28" t="inlineStr">
+        <is>
+          <t>No eligible registered case-count series facts are available for this disease and country; the public curve uses the legacy flat table.</t>
+        </is>
       </c>
       <c r="AV28" t="inlineStr">
         <is>
@@ -5101,6 +5356,11 @@
       <c r="Q29" t="n">
         <v>0</v>
       </c>
+      <c r="S29" t="inlineStr">
+        <is>
+          <t>missing_population</t>
+        </is>
+      </c>
       <c r="AA29" t="inlineStr">
         <is>
           <t>monthly</t>
@@ -5113,12 +5373,22 @@
       </c>
       <c r="AP29" t="inlineStr">
         <is>
-          <t>published_series</t>
+          <t>legacy_fallback</t>
+        </is>
+      </c>
+      <c r="AR29" t="inlineStr">
+        <is>
+          <t>legacy_identity_may_be_lossy</t>
         </is>
       </c>
       <c r="AS29" t="inlineStr"/>
       <c r="AT29" t="n">
         <v>0</v>
+      </c>
+      <c r="AU29" t="inlineStr">
+        <is>
+          <t>No eligible registered case-count series facts are available for this disease and country; the public curve uses the legacy flat table.</t>
+        </is>
       </c>
       <c r="AV29" t="inlineStr">
         <is>
@@ -5236,6 +5506,11 @@
       <c r="Q30" t="n">
         <v>0</v>
       </c>
+      <c r="S30" t="inlineStr">
+        <is>
+          <t>missing_population</t>
+        </is>
+      </c>
       <c r="AA30" t="inlineStr">
         <is>
           <t>monthly</t>
@@ -5248,12 +5523,22 @@
       </c>
       <c r="AP30" t="inlineStr">
         <is>
-          <t>published_series</t>
+          <t>legacy_fallback</t>
+        </is>
+      </c>
+      <c r="AR30" t="inlineStr">
+        <is>
+          <t>legacy_identity_may_be_lossy</t>
         </is>
       </c>
       <c r="AS30" t="inlineStr"/>
       <c r="AT30" t="n">
         <v>0</v>
+      </c>
+      <c r="AU30" t="inlineStr">
+        <is>
+          <t>No eligible registered case-count series facts are available for this disease and country; the public curve uses the legacy flat table.</t>
+        </is>
       </c>
       <c r="AV30" t="inlineStr">
         <is>
@@ -5371,6 +5656,11 @@
       <c r="Q31" t="n">
         <v>0</v>
       </c>
+      <c r="S31" t="inlineStr">
+        <is>
+          <t>missing_population</t>
+        </is>
+      </c>
       <c r="AA31" t="inlineStr">
         <is>
           <t>monthly</t>
@@ -5383,12 +5673,22 @@
       </c>
       <c r="AP31" t="inlineStr">
         <is>
-          <t>published_series</t>
+          <t>legacy_fallback</t>
+        </is>
+      </c>
+      <c r="AR31" t="inlineStr">
+        <is>
+          <t>legacy_identity_may_be_lossy</t>
         </is>
       </c>
       <c r="AS31" t="inlineStr"/>
       <c r="AT31" t="n">
         <v>0</v>
+      </c>
+      <c r="AU31" t="inlineStr">
+        <is>
+          <t>No eligible registered case-count series facts are available for this disease and country; the public curve uses the legacy flat table.</t>
+        </is>
       </c>
       <c r="AV31" t="inlineStr">
         <is>
@@ -5506,6 +5806,11 @@
       <c r="Q32" t="n">
         <v>0</v>
       </c>
+      <c r="S32" t="inlineStr">
+        <is>
+          <t>missing_population</t>
+        </is>
+      </c>
       <c r="AA32" t="inlineStr">
         <is>
           <t>monthly</t>
@@ -5518,12 +5823,22 @@
       </c>
       <c r="AP32" t="inlineStr">
         <is>
-          <t>published_series</t>
+          <t>legacy_fallback</t>
+        </is>
+      </c>
+      <c r="AR32" t="inlineStr">
+        <is>
+          <t>legacy_identity_may_be_lossy</t>
         </is>
       </c>
       <c r="AS32" t="inlineStr"/>
       <c r="AT32" t="n">
         <v>0</v>
+      </c>
+      <c r="AU32" t="inlineStr">
+        <is>
+          <t>No eligible registered case-count series facts are available for this disease and country; the public curve uses the legacy flat table.</t>
+        </is>
       </c>
       <c r="AV32" t="inlineStr">
         <is>
@@ -5641,6 +5956,11 @@
       <c r="Q33" t="n">
         <v>0</v>
       </c>
+      <c r="S33" t="inlineStr">
+        <is>
+          <t>missing_population</t>
+        </is>
+      </c>
       <c r="AA33" t="inlineStr">
         <is>
           <t>monthly</t>
@@ -5653,12 +5973,22 @@
       </c>
       <c r="AP33" t="inlineStr">
         <is>
-          <t>published_series</t>
+          <t>legacy_fallback</t>
+        </is>
+      </c>
+      <c r="AR33" t="inlineStr">
+        <is>
+          <t>legacy_identity_may_be_lossy</t>
         </is>
       </c>
       <c r="AS33" t="inlineStr"/>
       <c r="AT33" t="n">
         <v>0</v>
+      </c>
+      <c r="AU33" t="inlineStr">
+        <is>
+          <t>No eligible registered case-count series facts are available for this disease and country; the public curve uses the legacy flat table.</t>
+        </is>
       </c>
       <c r="AV33" t="inlineStr">
         <is>
@@ -5776,6 +6106,11 @@
       <c r="Q34" t="n">
         <v>0</v>
       </c>
+      <c r="S34" t="inlineStr">
+        <is>
+          <t>missing_population</t>
+        </is>
+      </c>
       <c r="AA34" t="inlineStr">
         <is>
           <t>monthly</t>
@@ -5788,12 +6123,22 @@
       </c>
       <c r="AP34" t="inlineStr">
         <is>
-          <t>published_series</t>
+          <t>legacy_fallback</t>
+        </is>
+      </c>
+      <c r="AR34" t="inlineStr">
+        <is>
+          <t>legacy_identity_may_be_lossy</t>
         </is>
       </c>
       <c r="AS34" t="inlineStr"/>
       <c r="AT34" t="n">
         <v>0</v>
+      </c>
+      <c r="AU34" t="inlineStr">
+        <is>
+          <t>No eligible registered case-count series facts are available for this disease and country; the public curve uses the legacy flat table.</t>
+        </is>
       </c>
       <c r="AV34" t="inlineStr">
         <is>
@@ -5911,6 +6256,11 @@
       <c r="Q35" t="n">
         <v>0</v>
       </c>
+      <c r="S35" t="inlineStr">
+        <is>
+          <t>missing_population</t>
+        </is>
+      </c>
       <c r="AA35" t="inlineStr">
         <is>
           <t>monthly</t>
@@ -5923,12 +6273,22 @@
       </c>
       <c r="AP35" t="inlineStr">
         <is>
-          <t>published_series</t>
+          <t>legacy_fallback</t>
+        </is>
+      </c>
+      <c r="AR35" t="inlineStr">
+        <is>
+          <t>legacy_identity_may_be_lossy</t>
         </is>
       </c>
       <c r="AS35" t="inlineStr"/>
       <c r="AT35" t="n">
         <v>0</v>
+      </c>
+      <c r="AU35" t="inlineStr">
+        <is>
+          <t>No eligible registered case-count series facts are available for this disease and country; the public curve uses the legacy flat table.</t>
+        </is>
       </c>
       <c r="AV35" t="inlineStr">
         <is>
@@ -6436,6 +6796,11 @@
       <c r="Q38" t="n">
         <v>0</v>
       </c>
+      <c r="S38" t="inlineStr">
+        <is>
+          <t>missing_population</t>
+        </is>
+      </c>
       <c r="AA38" t="inlineStr">
         <is>
           <t>monthly</t>
@@ -6448,12 +6813,22 @@
       </c>
       <c r="AP38" t="inlineStr">
         <is>
-          <t>published_series</t>
+          <t>legacy_fallback</t>
+        </is>
+      </c>
+      <c r="AR38" t="inlineStr">
+        <is>
+          <t>legacy_identity_may_be_lossy</t>
         </is>
       </c>
       <c r="AS38" t="inlineStr"/>
       <c r="AT38" t="n">
         <v>0</v>
+      </c>
+      <c r="AU38" t="inlineStr">
+        <is>
+          <t>No eligible registered case-count series facts are available for this disease and country; the public curve uses the legacy flat table.</t>
+        </is>
       </c>
       <c r="AV38" t="inlineStr">
         <is>
@@ -6810,6 +7185,11 @@
       <c r="Q40" t="n">
         <v>0</v>
       </c>
+      <c r="S40" t="inlineStr">
+        <is>
+          <t>missing_population</t>
+        </is>
+      </c>
       <c r="AA40" t="inlineStr">
         <is>
           <t>monthly</t>
@@ -6822,12 +7202,22 @@
       </c>
       <c r="AP40" t="inlineStr">
         <is>
-          <t>published_series</t>
+          <t>legacy_fallback</t>
+        </is>
+      </c>
+      <c r="AR40" t="inlineStr">
+        <is>
+          <t>legacy_identity_may_be_lossy</t>
         </is>
       </c>
       <c r="AS40" t="inlineStr"/>
       <c r="AT40" t="n">
         <v>0</v>
+      </c>
+      <c r="AU40" t="inlineStr">
+        <is>
+          <t>No eligible registered case-count series facts are available for this disease and country; the public curve uses the legacy flat table.</t>
+        </is>
       </c>
       <c r="AV40" t="inlineStr">
         <is>
@@ -6945,6 +7335,11 @@
       <c r="Q41" t="n">
         <v>0</v>
       </c>
+      <c r="S41" t="inlineStr">
+        <is>
+          <t>missing_population</t>
+        </is>
+      </c>
       <c r="AA41" t="inlineStr">
         <is>
           <t>monthly</t>
@@ -6957,12 +7352,22 @@
       </c>
       <c r="AP41" t="inlineStr">
         <is>
-          <t>published_series</t>
+          <t>legacy_fallback</t>
+        </is>
+      </c>
+      <c r="AR41" t="inlineStr">
+        <is>
+          <t>legacy_identity_may_be_lossy</t>
         </is>
       </c>
       <c r="AS41" t="inlineStr"/>
       <c r="AT41" t="n">
         <v>0</v>
+      </c>
+      <c r="AU41" t="inlineStr">
+        <is>
+          <t>No eligible registered case-count series facts are available for this disease and country; the public curve uses the legacy flat table.</t>
+        </is>
       </c>
       <c r="AV41" t="inlineStr">
         <is>
@@ -7080,6 +7485,11 @@
       <c r="Q42" t="n">
         <v>0</v>
       </c>
+      <c r="S42" t="inlineStr">
+        <is>
+          <t>missing_population</t>
+        </is>
+      </c>
       <c r="AA42" t="inlineStr">
         <is>
           <t>monthly</t>
@@ -7092,12 +7502,22 @@
       </c>
       <c r="AP42" t="inlineStr">
         <is>
-          <t>published_series</t>
+          <t>legacy_fallback</t>
+        </is>
+      </c>
+      <c r="AR42" t="inlineStr">
+        <is>
+          <t>legacy_identity_may_be_lossy</t>
         </is>
       </c>
       <c r="AS42" t="inlineStr"/>
       <c r="AT42" t="n">
         <v>0</v>
+      </c>
+      <c r="AU42" t="inlineStr">
+        <is>
+          <t>No eligible registered case-count series facts are available for this disease and country; the public curve uses the legacy flat table.</t>
+        </is>
       </c>
       <c r="AV42" t="inlineStr">
         <is>
@@ -7215,6 +7635,11 @@
       <c r="Q43" t="n">
         <v>0</v>
       </c>
+      <c r="S43" t="inlineStr">
+        <is>
+          <t>missing_population</t>
+        </is>
+      </c>
       <c r="AA43" t="inlineStr">
         <is>
           <t>monthly</t>
@@ -7227,12 +7652,22 @@
       </c>
       <c r="AP43" t="inlineStr">
         <is>
-          <t>published_series</t>
+          <t>legacy_fallback</t>
+        </is>
+      </c>
+      <c r="AR43" t="inlineStr">
+        <is>
+          <t>legacy_identity_may_be_lossy</t>
         </is>
       </c>
       <c r="AS43" t="inlineStr"/>
       <c r="AT43" t="n">
         <v>0</v>
+      </c>
+      <c r="AU43" t="inlineStr">
+        <is>
+          <t>No eligible registered case-count series facts are available for this disease and country; the public curve uses the legacy flat table.</t>
+        </is>
       </c>
       <c r="AV43" t="inlineStr">
         <is>
@@ -7350,6 +7785,11 @@
       <c r="Q44" t="n">
         <v>0</v>
       </c>
+      <c r="S44" t="inlineStr">
+        <is>
+          <t>missing_population</t>
+        </is>
+      </c>
       <c r="AA44" t="inlineStr">
         <is>
           <t>monthly</t>
@@ -7362,12 +7802,22 @@
       </c>
       <c r="AP44" t="inlineStr">
         <is>
-          <t>published_series</t>
+          <t>legacy_fallback</t>
+        </is>
+      </c>
+      <c r="AR44" t="inlineStr">
+        <is>
+          <t>legacy_identity_may_be_lossy</t>
         </is>
       </c>
       <c r="AS44" t="inlineStr"/>
       <c r="AT44" t="n">
         <v>0</v>
+      </c>
+      <c r="AU44" t="inlineStr">
+        <is>
+          <t>No eligible registered case-count series facts are available for this disease and country; the public curve uses the legacy flat table.</t>
+        </is>
       </c>
       <c r="AV44" t="inlineStr">
         <is>
@@ -7485,6 +7935,11 @@
       <c r="Q45" t="n">
         <v>0</v>
       </c>
+      <c r="S45" t="inlineStr">
+        <is>
+          <t>missing_population</t>
+        </is>
+      </c>
       <c r="AA45" t="inlineStr">
         <is>
           <t>monthly</t>
@@ -7497,12 +7952,22 @@
       </c>
       <c r="AP45" t="inlineStr">
         <is>
-          <t>published_series</t>
+          <t>legacy_fallback</t>
+        </is>
+      </c>
+      <c r="AR45" t="inlineStr">
+        <is>
+          <t>legacy_identity_may_be_lossy</t>
         </is>
       </c>
       <c r="AS45" t="inlineStr"/>
       <c r="AT45" t="n">
         <v>0</v>
+      </c>
+      <c r="AU45" t="inlineStr">
+        <is>
+          <t>No eligible registered case-count series facts are available for this disease and country; the public curve uses the legacy flat table.</t>
+        </is>
       </c>
       <c r="AV45" t="inlineStr">
         <is>
@@ -7620,6 +8085,11 @@
       <c r="Q46" t="n">
         <v>0</v>
       </c>
+      <c r="S46" t="inlineStr">
+        <is>
+          <t>missing_population</t>
+        </is>
+      </c>
       <c r="AA46" t="inlineStr">
         <is>
           <t>monthly</t>
@@ -7632,12 +8102,22 @@
       </c>
       <c r="AP46" t="inlineStr">
         <is>
-          <t>published_series</t>
+          <t>legacy_fallback</t>
+        </is>
+      </c>
+      <c r="AR46" t="inlineStr">
+        <is>
+          <t>legacy_identity_may_be_lossy</t>
         </is>
       </c>
       <c r="AS46" t="inlineStr"/>
       <c r="AT46" t="n">
         <v>0</v>
+      </c>
+      <c r="AU46" t="inlineStr">
+        <is>
+          <t>No eligible registered case-count series facts are available for this disease and country; the public curve uses the legacy flat table.</t>
+        </is>
       </c>
       <c r="AV46" t="inlineStr">
         <is>
@@ -7755,6 +8235,11 @@
       <c r="Q47" t="n">
         <v>0</v>
       </c>
+      <c r="S47" t="inlineStr">
+        <is>
+          <t>missing_population</t>
+        </is>
+      </c>
       <c r="AA47" t="inlineStr">
         <is>
           <t>monthly</t>
@@ -7767,12 +8252,22 @@
       </c>
       <c r="AP47" t="inlineStr">
         <is>
-          <t>published_series</t>
+          <t>legacy_fallback</t>
+        </is>
+      </c>
+      <c r="AR47" t="inlineStr">
+        <is>
+          <t>legacy_identity_may_be_lossy</t>
         </is>
       </c>
       <c r="AS47" t="inlineStr"/>
       <c r="AT47" t="n">
         <v>0</v>
+      </c>
+      <c r="AU47" t="inlineStr">
+        <is>
+          <t>No eligible registered case-count series facts are available for this disease and country; the public curve uses the legacy flat table.</t>
+        </is>
       </c>
       <c r="AV47" t="inlineStr">
         <is>
@@ -7890,6 +8385,11 @@
       <c r="Q48" t="n">
         <v>0</v>
       </c>
+      <c r="S48" t="inlineStr">
+        <is>
+          <t>missing_population</t>
+        </is>
+      </c>
       <c r="AA48" t="inlineStr">
         <is>
           <t>monthly</t>
@@ -7902,12 +8402,22 @@
       </c>
       <c r="AP48" t="inlineStr">
         <is>
-          <t>published_series</t>
+          <t>legacy_fallback</t>
+        </is>
+      </c>
+      <c r="AR48" t="inlineStr">
+        <is>
+          <t>legacy_identity_may_be_lossy</t>
         </is>
       </c>
       <c r="AS48" t="inlineStr"/>
       <c r="AT48" t="n">
         <v>0</v>
+      </c>
+      <c r="AU48" t="inlineStr">
+        <is>
+          <t>No eligible registered case-count series facts are available for this disease and country; the public curve uses the legacy flat table.</t>
+        </is>
       </c>
       <c r="AV48" t="inlineStr">
         <is>
@@ -8025,6 +8535,11 @@
       <c r="Q49" t="n">
         <v>0</v>
       </c>
+      <c r="S49" t="inlineStr">
+        <is>
+          <t>missing_population</t>
+        </is>
+      </c>
       <c r="AA49" t="inlineStr">
         <is>
           <t>monthly</t>
@@ -8037,12 +8552,22 @@
       </c>
       <c r="AP49" t="inlineStr">
         <is>
-          <t>published_series</t>
+          <t>legacy_fallback</t>
+        </is>
+      </c>
+      <c r="AR49" t="inlineStr">
+        <is>
+          <t>legacy_identity_may_be_lossy</t>
         </is>
       </c>
       <c r="AS49" t="inlineStr"/>
       <c r="AT49" t="n">
         <v>0</v>
+      </c>
+      <c r="AU49" t="inlineStr">
+        <is>
+          <t>No eligible registered case-count series facts are available for this disease and country; the public curve uses the legacy flat table.</t>
+        </is>
       </c>
       <c r="AV49" t="inlineStr">
         <is>
@@ -8160,6 +8685,11 @@
       <c r="Q50" t="n">
         <v>0</v>
       </c>
+      <c r="S50" t="inlineStr">
+        <is>
+          <t>missing_population</t>
+        </is>
+      </c>
       <c r="AA50" t="inlineStr">
         <is>
           <t>monthly</t>
@@ -8172,12 +8702,22 @@
       </c>
       <c r="AP50" t="inlineStr">
         <is>
-          <t>published_series</t>
+          <t>legacy_fallback</t>
+        </is>
+      </c>
+      <c r="AR50" t="inlineStr">
+        <is>
+          <t>legacy_identity_may_be_lossy</t>
         </is>
       </c>
       <c r="AS50" t="inlineStr"/>
       <c r="AT50" t="n">
         <v>0</v>
+      </c>
+      <c r="AU50" t="inlineStr">
+        <is>
+          <t>No eligible registered case-count series facts are available for this disease and country; the public curve uses the legacy flat table.</t>
+        </is>
       </c>
       <c r="AV50" t="inlineStr">
         <is>

</xml_diff>